<commit_message>
[TEST] Added tests for postUploadXlsxDependencies.
</commit_message>
<xml_diff>
--- a/src/__tests__/notifications/__testFiles__/Modifica Dependencias.xlsx
+++ b/src/__tests__/notifications/__testFiles__/Modifica Dependencias.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,32 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TBBC\Proyectos\Cali Movilidad\cali-mobility-backend\src\__tests__\notifications\__testFiles__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{12D7B16E-5305-4AB4-8BB1-2014F3C7B40B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99437399-A0ED-4994-8AEB-12B1959E9A74}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>JuLiAnChO... PlZSs</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -71,7 +63,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -152,7 +144,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -487,7 +479,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -505,7 +497,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -513,7 +505,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -521,7 +513,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>

</xml_diff>